<commit_message>
Restore full oracle price history after accidental truncate.
Recovered 2048 mark samples (seed-walk + dual-source) from the last good
git revision; harden appendPriceSamples so a corrupt/empty read cannot
wipe thousands of samples on the next cron push.
</commit_message>
<xml_diff>
--- a/frontend/public/data/price-history.xlsx
+++ b/frontend/public/data/price-history.xlsx
@@ -15,11 +15,11 @@
     <sheet name="GLP1-IDX-PERP" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Samples'!$A$1:$F$2046</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SEMA-PERP'!$A$1:$E$522</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Samples'!$A$1:$F$2052</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SEMA-PERP'!$A$1:$E$524</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TIRZ-PERP'!$A$1:$E$483</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RETA-PERP'!$A$1:$E$522</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'GLP1-IDX-PERP'!$A$1:$E$522</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RETA-PERP'!$A$1:$E$524</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'GLP1-IDX-PERP'!$A$1:$E$524</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -243,7 +243,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'SEMA-PERP'!$B$2:$B$522</f>
+              <f>'SEMA-PERP'!$B$2:$B$524</f>
             </numRef>
           </val>
         </ser>
@@ -471,7 +471,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'RETA-PERP'!$B$2:$B$522</f>
+              <f>'RETA-PERP'!$B$2:$B$524</f>
             </numRef>
           </val>
         </ser>
@@ -585,7 +585,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'GLP1-IDX-PERP'!$B$2:$B$522</f>
+              <f>'GLP1-IDX-PERP'!$B$2:$B$524</f>
             </numRef>
           </val>
         </ser>
@@ -1075,14 +1075,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Exported 2026-07-18 08:31 UTC · source updatedAt=2026-07-18T08:23:13.529Z</t>
+          <t>Exported 2026-07-18 08:35 UTC · source updatedAt=2026-07-18T08:35:18.951Z</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Oracle mark samples for PEPT Trade charts. Appended on each successful pushPrice (~5m cron). Fine TFs (5m/15m) need dense samples; coarser TFs still stair-step when marks are quiet.</t>
+          <t>Oracle mark samples for PEPT Trade charts. Appended on each successful pushPrice (~5m cron). Fine TFs (5m/15m) need dense samples; coarser TFs still stair-step when marks are quiet. Full history restored 2026-07-18 (seed-walk + dual-source marks; not wiped by vendor expansion).</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -1165,14 +1165,14 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-18 08:23</t>
+          <t>2026-07-18 08:33</t>
         </is>
       </c>
       <c r="E9" s="8" t="n">
         <v>4.949</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.8213</v>
+        <v>5.6584</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>4.0963</v>
@@ -1181,7 +1181,7 @@
         <v>5.8213</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>0.1762578298646191</v>
+        <v>0.143342089310972</v>
       </c>
     </row>
     <row r="10">
@@ -1226,7 +1226,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -1235,14 +1235,14 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-18 08:23</t>
+          <t>2026-07-18 08:33</t>
         </is>
       </c>
       <c r="E11" s="8" t="n">
         <v>4.9112</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>5.3325</v>
+        <v>5.1629</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>4.8665</v>
@@ -1251,7 +1251,7 @@
         <v>5.5878</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.08578351523049348</v>
+        <v>0.05125020361622406</v>
       </c>
     </row>
     <row r="12">
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="B12" s="11" t="n">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
@@ -1270,14 +1270,14 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>2026-07-18 08:23</t>
+          <t>2026-07-18 08:33</t>
         </is>
       </c>
       <c r="E12" s="12" t="n">
         <v>4.5765</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>5.1738</v>
+        <v>5.0491</v>
       </c>
       <c r="G12" s="12" t="n">
         <v>4.0787</v>
@@ -1286,7 +1286,7 @@
         <v>5.1738</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>0.130514585381842</v>
+        <v>0.103266688517426</v>
       </c>
     </row>
     <row r="13"/>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>2045</v>
+        <v>2051</v>
       </c>
     </row>
   </sheetData>
@@ -1315,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2046"/>
+  <dimension ref="A1:F2052"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -46816,8 +46816,164 @@
         </is>
       </c>
     </row>
+    <row r="2047">
+      <c r="A2047" s="6" t="inlineStr">
+        <is>
+          <t>GLP1-IDX-PERP</t>
+        </is>
+      </c>
+      <c r="B2047" s="7" t="n">
+        <v>1784363115</v>
+      </c>
+      <c r="C2047" s="15" t="n">
+        <v>46221.35086805555</v>
+      </c>
+      <c r="D2047" s="8" t="n">
+        <v>5.1738</v>
+      </c>
+      <c r="E2047" s="6" t="inlineStr">
+        <is>
+          <t>Weighted 60% SEMA / 25% TIRZ / 15% RETA · dual-source medians</t>
+        </is>
+      </c>
+      <c r="F2047" s="6" t="inlineStr">
+        <is>
+          <t>0x12d62769c0e4a3886c774691f1e69ab49e3e06f529f646669a94ac606ea599ee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" s="10" t="inlineStr">
+        <is>
+          <t>RETA-PERP</t>
+        </is>
+      </c>
+      <c r="B2048" s="11" t="n">
+        <v>1784363115</v>
+      </c>
+      <c r="C2048" s="14" t="n">
+        <v>46221.35086805555</v>
+      </c>
+      <c r="D2048" s="12" t="n">
+        <v>5.3325</v>
+      </c>
+      <c r="E2048" s="10" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.7412(n=92) · vendor_basket=$6.2961(n=69) · divergence=32.8%</t>
+        </is>
+      </c>
+      <c r="F2048" s="10" t="inlineStr">
+        <is>
+          <t>0x85e05e5b2c1f4569be4f268a70432143df17f56e5b8b1bd3e48e8e931474f43c</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" s="6" t="inlineStr">
+        <is>
+          <t>SEMA-PERP</t>
+        </is>
+      </c>
+      <c r="B2049" s="7" t="n">
+        <v>1784363115</v>
+      </c>
+      <c r="C2049" s="15" t="n">
+        <v>46221.35086805555</v>
+      </c>
+      <c r="D2049" s="8" t="n">
+        <v>5.8213</v>
+      </c>
+      <c r="E2049" s="6" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.3791(n=27) · vendor_basket=$7.1811(n=35) · divergence=64.0%</t>
+        </is>
+      </c>
+      <c r="F2049" s="6" t="inlineStr">
+        <is>
+          <t>0x82340951b1d47a776789a0df2159960b587f79e97a6ecfdaa200af64c0e350e4</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" s="10" t="inlineStr">
+        <is>
+          <t>GLP1-IDX-PERP</t>
+        </is>
+      </c>
+      <c r="B2050" s="11" t="n">
+        <v>1784363625</v>
+      </c>
+      <c r="C2050" s="14" t="n">
+        <v>46221.35677083334</v>
+      </c>
+      <c r="D2050" s="12" t="n">
+        <v>5.0491</v>
+      </c>
+      <c r="E2050" s="10" t="inlineStr">
+        <is>
+          <t>Weighted 60% SEMA / 25% TIRZ / 15% RETA · dual-source medians</t>
+        </is>
+      </c>
+      <c r="F2050" s="10" t="inlineStr">
+        <is>
+          <t>0x397ed7dbc0c84c3768ff4f757d03ae8e386e296fe0f1108b2fcea62df228f49e</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" s="6" t="inlineStr">
+        <is>
+          <t>RETA-PERP</t>
+        </is>
+      </c>
+      <c r="B2051" s="7" t="n">
+        <v>1784363625</v>
+      </c>
+      <c r="C2051" s="15" t="n">
+        <v>46221.35677083334</v>
+      </c>
+      <c r="D2051" s="8" t="n">
+        <v>5.1629</v>
+      </c>
+      <c r="E2051" s="6" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.7412(n=92) · vendor_basket=$5.9947(n=57) · divergence=26.4%</t>
+        </is>
+      </c>
+      <c r="F2051" s="6" t="inlineStr">
+        <is>
+          <t>0x9c618cb05318184b5d4562205dea1b879b3d8884a74001c4c3974cfdfcc50663</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" s="10" t="inlineStr">
+        <is>
+          <t>SEMA-PERP</t>
+        </is>
+      </c>
+      <c r="B2052" s="11" t="n">
+        <v>1784363625</v>
+      </c>
+      <c r="C2052" s="14" t="n">
+        <v>46221.35677083334</v>
+      </c>
+      <c r="D2052" s="12" t="n">
+        <v>5.6584</v>
+      </c>
+      <c r="E2052" s="10" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.3791(n=27) · vendor_basket=$7.0656(n=30) · divergence=61.4%</t>
+        </is>
+      </c>
+      <c r="F2052" s="10" t="inlineStr">
+        <is>
+          <t>0x47852bcf26163ff942af76b0d77f7785834990caffe0dce7401104f497b1a020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F2046"/>
+  <autoFilter ref="A1:F2052"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -46828,7 +46984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E522"/>
+  <dimension ref="A1:E524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -55878,8 +56034,50 @@
         <v>1784362987</v>
       </c>
     </row>
+    <row r="523">
+      <c r="A523" s="15" t="n">
+        <v>46221.35086805555</v>
+      </c>
+      <c r="B523" s="8" t="n">
+        <v>5.8213</v>
+      </c>
+      <c r="C523" s="6" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.3791(n=27) · vendor_basket=$7.1811(n=35) · divergence=64.0%</t>
+        </is>
+      </c>
+      <c r="D523" s="6" t="inlineStr">
+        <is>
+          <t>0x82340951b1d47a776789a0df2159960b587f79e97a6ecfdaa200af64c0e350e4</t>
+        </is>
+      </c>
+      <c r="E523" s="6" t="n">
+        <v>1784363115</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="15" t="n">
+        <v>46221.35677083334</v>
+      </c>
+      <c r="B524" s="8" t="n">
+        <v>5.6584</v>
+      </c>
+      <c r="C524" s="6" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.3791(n=27) · vendor_basket=$7.0656(n=30) · divergence=61.4%</t>
+        </is>
+      </c>
+      <c r="D524" s="6" t="inlineStr">
+        <is>
+          <t>0x47852bcf26163ff942af76b0d77f7785834990caffe0dce7401104f497b1a020</t>
+        </is>
+      </c>
+      <c r="E524" s="6" t="n">
+        <v>1784363625</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E522"/>
+  <autoFilter ref="A1:E524"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -64135,7 +64333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E522"/>
+  <dimension ref="A1:E524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -73185,8 +73383,50 @@
         <v>1784362987</v>
       </c>
     </row>
+    <row r="523">
+      <c r="A523" s="15" t="n">
+        <v>46221.35086805555</v>
+      </c>
+      <c r="B523" s="8" t="n">
+        <v>5.3325</v>
+      </c>
+      <c r="C523" s="6" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.7412(n=92) · vendor_basket=$6.2961(n=69) · divergence=32.8%</t>
+        </is>
+      </c>
+      <c r="D523" s="6" t="inlineStr">
+        <is>
+          <t>0x85e05e5b2c1f4569be4f268a70432143df17f56e5b8b1bd3e48e8e931474f43c</t>
+        </is>
+      </c>
+      <c r="E523" s="6" t="n">
+        <v>1784363115</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="15" t="n">
+        <v>46221.35677083334</v>
+      </c>
+      <c r="B524" s="8" t="n">
+        <v>5.1629</v>
+      </c>
+      <c r="C524" s="6" t="inlineStr">
+        <is>
+          <t>Dual source weighted · peptidescouter=$4.7412(n=92) · vendor_basket=$5.9947(n=57) · divergence=26.4%</t>
+        </is>
+      </c>
+      <c r="D524" s="6" t="inlineStr">
+        <is>
+          <t>0x9c618cb05318184b5d4562205dea1b879b3d8884a74001c4c3974cfdfcc50663</t>
+        </is>
+      </c>
+      <c r="E524" s="6" t="n">
+        <v>1784363625</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E522"/>
+  <autoFilter ref="A1:E524"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -73198,7 +73438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E522"/>
+  <dimension ref="A1:E524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -82248,8 +82488,50 @@
         <v>1784362987</v>
       </c>
     </row>
+    <row r="523">
+      <c r="A523" s="15" t="n">
+        <v>46221.35086805555</v>
+      </c>
+      <c r="B523" s="8" t="n">
+        <v>5.1738</v>
+      </c>
+      <c r="C523" s="6" t="inlineStr">
+        <is>
+          <t>Weighted 60% SEMA / 25% TIRZ / 15% RETA · dual-source medians</t>
+        </is>
+      </c>
+      <c r="D523" s="6" t="inlineStr">
+        <is>
+          <t>0x12d62769c0e4a3886c774691f1e69ab49e3e06f529f646669a94ac606ea599ee</t>
+        </is>
+      </c>
+      <c r="E523" s="6" t="n">
+        <v>1784363115</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="15" t="n">
+        <v>46221.35677083334</v>
+      </c>
+      <c r="B524" s="8" t="n">
+        <v>5.0491</v>
+      </c>
+      <c r="C524" s="6" t="inlineStr">
+        <is>
+          <t>Weighted 60% SEMA / 25% TIRZ / 15% RETA · dual-source medians</t>
+        </is>
+      </c>
+      <c r="D524" s="6" t="inlineStr">
+        <is>
+          <t>0x397ed7dbc0c84c3768ff4f757d03ae8e386e296fe0f1108b2fcea62df228f49e</t>
+        </is>
+      </c>
+      <c r="E524" s="6" t="n">
+        <v>1784363625</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E522"/>
+  <autoFilter ref="A1:E524"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>